<commit_message>
Implement Cinema Mode layout, diagnose Sony Pix CORS issue, and complete 80-stream playback audit
</commit_message>
<xml_diff>
--- a/05_STREAMING_PORTAL/IPTV_Playlist_Merged_Primary.xlsx
+++ b/05_STREAMING_PORTAL/IPTV_Playlist_Merged_Primary.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,40 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00155724"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001A1D20"/>
-        <bgColor rgb="001A1D20"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -66,35 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,2196 +415,2189 @@
   </sheetPr>
   <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="193" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>STREAM NAME</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CATEGORY</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ICON</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>7s Music Tv</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>https://cdn.pishow.tv/ott/live/1257/master.m3u8</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>🎵</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Aaryaa Tv</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>https://stream.ottlive.co.in/aryatvtamil/index.m3u8</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Aaseervatham TV</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>https://mumt04.tangotv.in/m18aqlK4AASEERVATHAMTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Aastha Tamil</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>https://aasthaott.akamaized.net/110923/smil:aasthatamil.smil/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Angel TV Indo-China</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>https://janya-digimix.akamaized.net/vglive-sk-703035/indochina/ngrp:angelindochina_all/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Arputhar Yesu TV</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>https://account33.livebox.co.in/jesushelpshls/live.m3u8</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Colors Tamil HD</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:colorstamilhd11.smil/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>✨</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Dharsan TV</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>https://cable91tataplay.akamaized.net/live/dharshantv/index.m3u8</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>ETV Bal Bharat</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>http://103.185.24.134:3001/ETV-BAL-BHARAT/index.m3u8</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Fail Army</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>https://failarmy-international-in.samsung.wurl.tv/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>🌐</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Hebron TV</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>https://account20.livebox.co.in/charleshls/live.m3u8</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Hosanna TV</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>https://asia.mslivestream.net/mslive/bfba54c5c96a6359e2da0ca35f4998af.sdp/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Hungama TV</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>http://103.185.24.134:3001/HUNGAMA/index.m3u8</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Isaiaruvi Tv</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>https://segment.yuppcdn.net/140622/isaiaruvi/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Joy TV</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>https://ktismaservers.in:3412/live/joytvlive.m3u8</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Kalaignar Murasu</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>https://yuppmedtaorire.akamaized.net/v1/master/a0d007312bfd99c47f76b77ae26b1ccdaae76cb1/murasu_nim_https/050522/murasu/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Kalaignar Tv</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>https://segment.yuppcdn.net/240122/kalaignartv/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Life TV</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>https://lifetv.livebox.co.in/lifetvhls/lifetv.m3u8</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Madha TV</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>https://mumt07.tangotv.in/zHjX9OFlMADHATV/index.m3u8</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Madhimugam TV</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>https://mumt01.tangotv.in/O5aw8Zn3MATHIMUGAMTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Makkal TV (576i)</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>https://5k8q87azdy4v-hls-live.wmncdn.net/MAKKAL/271ddf829afeece44d8732757fba1a66.sdp/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Mei Alai TV</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>https://meialai.iptelevishion.com/meialai/2/index.m3u8</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>MK Six</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>https://mumt06.tangotv.in/qYyB8fXVMKSIX/index.m3u8</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>MN Tv</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>https://mntv.livebox.co.in/mntvhls/live.m3u8</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Movie Club 2 Tv</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>https://d3gnyty2vddhsg.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-ytipwjqub3kf8/TMC2_IN.m3u8?ads.ads_cdn=cf&amp;ads.cdn=cf</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Hindi</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>🎬</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Movie Club Tv</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>https://sis-global.prod.samsungtv.plus/v1/tvpprd/sc-mp2ar4ca425xo.m3u8</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Hindi</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>🎬</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Murasu Tv</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>https://segment.yuppcdn.net/050522/murasu/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>NDTV Good Times</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>https://amg01448-samsungin-ndtvgoodtimes-samsungin-ad-gp.amagi.tv/playlist/amg01448-samsungin-ndtvgoodtimes-samsungin/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>News 7 Tv</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>https://segment.yuppcdn.net/240122/news7/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>News Tamil 24x7</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>https://cdn.pishow.tv/ott/live/1433/master.m3u8</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>News18 Tamil Nadu</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>https://n18syndication.akamaized.net/bpk-tv/News18_Tamil_Nadu_NW18_MOB/output01/master.m3u8</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>NH Tamil Gold</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>https://d3arbp6l7f096k.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-gv6wgpbb4mgwk/playlist.m3u8?ads.ads_cdn=cf&amp;ads.app_domain=APP_DOMAIN&amp;ads.cdn=cf</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>🎬</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Nickelodeon</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>http://103.185.24.134:3001/NICK/index.m3u8</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Oli TV</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>https://live.olidigital.in/olitv/olitv/index.m3u8</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>OM TV</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>https://mumt01.tangotv.in/O5aw8Zn3OMTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Polimer TV</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>https://cdn.pishow.tv/ott/live/1241/master.m3u8</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Puthiya Thalaimurai</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>https://mumt07.tangotv.in/zHjX9OFlPUTHIYAEXPRESS/index.m3u8</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Puthuyugam TV</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>https://mumt04.tangotv.in/m18aqlK4PUTHUYUGAMTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Raj Digital Plus</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/RajTV_Digital_plus/master_1.m3u8</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t>🎬</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Roja TV1</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>https://live.rojatv.cloud/rojatv/rojatv/index.m3u8</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Roja TV2</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>https://stream.rojatv.cloud/rojatv/rojatv/index.m3u8</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Sai TV</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>https://mumt03.tangotv.in/Dsly5z3HSAITV/index.m3u8</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Sairam TV</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>https://mumt04.tangotv.in/m18aqlK4SAIRAMTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Sana Plus</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>https://mumbai-edge.smartplaytv.in/SanaPlusHD/index.m3u8</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
         <is>
           <t>🎵</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Sanaa Tv</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>https://vglivessai.akamaized.net/us/v1/master/611d79b11b77e2f571934fd80ca1413453772ac7/b6d9e864-ec16-410a-804d-ccf8f720bfaa/index.m3u8</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Sankara TV</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>https://mumt05.tangotv.in/87NeALx2SRISANKARA/index.m3u8</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Sirippoli TV1</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>https://segment.yuppcdn.net/240122/siripoli/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Sirippoli TV2</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>https://yuppmedtaorire.akamaized.net/v1/manifest/a0d007312bfd99c47f76b77ae26b1ccdaae76cb1/siripoli_nim_https/c4e6500f-ea05-4226-810e-2833ee0075ff/0.m3u8</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Sivan TV</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>https://sivantv.livebox.co.in/sivantvhls/sivan.m3u8</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Sonic</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>http://103.185.24.134:3001/SONIC/index.m3u8</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Sony BBC Earth HD</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>https://cloudplay-sonyliv.pages.dev/bbcearthhd.m3u8</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
         <is>
           <t>✨</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Sony pix HD</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>https://cloudplay-sonyliv.pages.dev/pixhd.m3u8</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>✨</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Sony Sports Ten 4</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>https://cloudplay-sonyliv.pages.dev/ten4.m3u8</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>🏏</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Sony Yay!</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>https://cloudplay-sonyliv.pages.dev/yay.m3u8</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>South Station Tv</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>https://cc-yw7ztecy8do3q.akamaized.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/cc-yw7ztecy8do3q/SS_IN.m3u8</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Hindi</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>🎬</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Star Vijay</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:starvijayuk.smil/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Subin Tv</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>https://stream.galaxyott.live/live/subintv/index.m3u8</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Super Hungama</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>http://103.185.24.134:3001/SUPER-HUNGAMA/index.m3u8</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>SVBC 2</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>https://player.mslivestream.net/tamil/ac206e74d75b285755ee4924df87d951.sdp/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Tamil Janam</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>https://mumt01.tangotv.in/O5aw8Zn3JANAMTVTAMIL/index.m3u8</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>Tamilan TV</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>https://mumt04.tangotv.in/m18aqlK4TAMILANTELEVISION/index.m3u8</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Thalaa Tv</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>https://streams2.sofast.tv/ptnr-yupptv/title-THALAA-TV-TAM/sofastplayout/981f8f06-782a-4962-b5e0-7dcccd65279c_0_HLS/manifest.m3u8</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>Thanthi Tv</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>https://streams.tangotv.in/THANTHITV/ORIGIN/index.m3u8</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
         <is>
           <t>📰</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>Tharun Movies</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>https://streaming.livebox.co.in/tharunmovieshls/live.m3u8</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>Toonami Movie</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>http://api.toonamiaftermath.com:3000/movies/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>🌐</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>Travelxp HD</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>https://amg00416-amg00416c9-samsung-in-4882.playouts.now.amagi.tv/playlist/amg00416-travelxp-travelxphd-samsungin/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
         <is>
           <t>🌍</t>
         </is>
       </c>
-      <c r="E67" s="3" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>TVI HD</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>https://live.cmr24.fm/TVI/HD/chunks.m3u8</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>Ultimate TV1</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>https://stream.ottlive.co.in/utvtamil/index.m3u8</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>Ultimate TV2</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>https://mumbai-edge.smartplaytv.in/utv/index.m3u8</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>Vaanavil Tv</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>https://6n3yope4d9ok-hls-live.5centscdn.com/vaanavil/TV.stream/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>Vasanth TV</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>https://mumt04.tangotv.in/m18aqlK4VASANTHTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>Velicham Tv</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>https://mumt05.tangotv.in/87NeALx2VALICHAMPLUS/index.m3u8</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
         <is>
           <t>☀️</t>
         </is>
       </c>
-      <c r="E73" s="3" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>Vendhar TV</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>https://mumt04.tangotv.in/m18aqlK4VENDHARTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>Village TV</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>https://live.villagetv.net/villagetv/hd/index.m3u8</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
         <is>
           <t>🪷</t>
         </is>
       </c>
-      <c r="E75" s="3" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>Win Tv</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>https://mumt06.tangotv.in/qYyB8fXVWINTV/index.m3u8</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>WOW Kidz Tamil</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>https://yuppparoriglin.akamaized.net/181224/smil:wowkidztam.smil/playlist.m3u8?hdnts=st=1735898689~exp=1835898688~acl=*~hmac=f5fe24724fe05481e3841f9eb5ab8efdee0a3dd83645ae9dcf45703f525bab7b</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
         <is>
           <t>👶</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>YET Max</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv2.m3u8</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
         <is>
           <t>🎵</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>YET TV</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv.m3u8</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>📺</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>Zee South Flix Tv</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>https://amg00862-amg00862c9-amgplt0173.playout.now3.amagi.tv/playlist/amg00862-amg00862c9-amgplt0173/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>Hindi</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>🎬</t>
         </is>
       </c>
-      <c r="E80" s="3" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>Zee Tamil HD</t>
         </is>
       </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:zeetamil1.smil/playlist.m3u8</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>✨</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>Live</t>
         </is>

</xml_diff>